<commit_message>
chore: update MultiCell-BMS-OverAllFrame.xlsx with new data
</commit_message>
<xml_diff>
--- a/MultiCell-BMS-OverAllFrame.xlsx
+++ b/MultiCell-BMS-OverAllFrame.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shreyas\Documents\MultiCell-BMS-FrameConfig\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shreyas\Documents\Python\Bytehound\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C56BB0E-2AA3-4C35-9063-9439BC80E22A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28B4EF9D-A72F-4D79-A0BE-13EAEE794CFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,29 +18,18 @@
     <sheet name="Variables" sheetId="3" r:id="rId3"/>
     <sheet name="Bitfields" sheetId="4" r:id="rId4"/>
     <sheet name="Enums" sheetId="5" r:id="rId5"/>
-    <sheet name="TxCommands" sheetId="6" r:id="rId6"/>
-    <sheet name="TxCommandFields" sheetId="7" r:id="rId7"/>
-    <sheet name="PollingSchedule" sheetId="8" r:id="rId8"/>
+    <sheet name="CalcGroups" sheetId="6" r:id="rId6"/>
+    <sheet name="TxCommands" sheetId="7" r:id="rId7"/>
+    <sheet name="TxCommandFields" sheetId="8" r:id="rId8"/>
+    <sheet name="PollingSchedule" sheetId="9" r:id="rId9"/>
+    <sheet name="SerialDefaults" sheetId="10" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="175">
   <si>
     <t>profile_name</t>
   </si>
@@ -63,6 +52,9 @@
     <t>length_meaning</t>
   </si>
   <si>
+    <t>length_byte_order</t>
+  </si>
+  <si>
     <t>crc_type</t>
   </si>
   <si>
@@ -72,15 +64,27 @@
     <t>crc_byte_order</t>
   </si>
   <si>
+    <t>crc_coverage</t>
+  </si>
+  <si>
     <t>footer_hex</t>
   </si>
   <si>
+    <t>escape_mode</t>
+  </si>
+  <si>
+    <t>raw_log_format</t>
+  </si>
+  <si>
     <t>inter_frame_delay_ms</t>
   </si>
   <si>
     <t>tx_pad_length</t>
   </si>
   <si>
+    <t>modbus_node_address</t>
+  </si>
+  <si>
     <t>enabled</t>
   </si>
   <si>
@@ -102,6 +106,18 @@
     <t>crc16_modbus</t>
   </si>
   <si>
+    <t>big</t>
+  </si>
+  <si>
+    <t>header_to_payload</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>hex</t>
+  </si>
+  <si>
     <t>TRUE</t>
   </si>
   <si>
@@ -123,15 +139,69 @@
     <t>0x1000</t>
   </si>
   <si>
+    <t>Pack Voltage &amp; Current</t>
+  </si>
+  <si>
     <t>rx</t>
   </si>
   <si>
     <t>0x2000</t>
   </si>
   <si>
+    <t>Cell Voltages</t>
+  </si>
+  <si>
     <t>0x3000</t>
   </si>
   <si>
+    <t>Pack Temperature Sensors</t>
+  </si>
+  <si>
+    <t>0x4000</t>
+  </si>
+  <si>
+    <t>Onboard Temperature Sensors</t>
+  </si>
+  <si>
+    <t>0x5000</t>
+  </si>
+  <si>
+    <t>BCC Fault Status</t>
+  </si>
+  <si>
+    <t>Array containing all fault status information provided by BCC</t>
+  </si>
+  <si>
+    <t>0x6000</t>
+  </si>
+  <si>
+    <t>Load Voltage</t>
+  </si>
+  <si>
+    <t>0x7000</t>
+  </si>
+  <si>
+    <t>Cell Balancing Status</t>
+  </si>
+  <si>
+    <t>0x8000</t>
+  </si>
+  <si>
+    <t>Fault Status</t>
+  </si>
+  <si>
+    <t>0x9000</t>
+  </si>
+  <si>
+    <t>FET Status</t>
+  </si>
+  <si>
+    <t>0x9001</t>
+  </si>
+  <si>
+    <t>Algorithm</t>
+  </si>
+  <si>
     <t>id_or_address</t>
   </si>
   <si>
@@ -186,28 +256,136 @@
     <t>Pack Current</t>
   </si>
   <si>
+    <t>int32</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Charge (+) / discharge (-) current</t>
+  </si>
+  <si>
+    <t>Cell Voltage</t>
+  </si>
+  <si>
+    <t>Series Cell Voltage</t>
+  </si>
+  <si>
+    <t>14 individual cell voltages expanded automatically</t>
+  </si>
+  <si>
+    <t>Pack Temperature</t>
+  </si>
+  <si>
     <t>int16</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Charge (+) / discharge (-) current</t>
-  </si>
-  <si>
-    <t>Pack Temperature</t>
-  </si>
-  <si>
     <t>°C</t>
   </si>
   <si>
     <t>Pack temperature sensor</t>
   </si>
   <si>
-    <t>Cell Voltage</t>
-  </si>
-  <si>
-    <t>Cell Voltages</t>
+    <t>Balancing Resistor Temperature</t>
+  </si>
+  <si>
+    <t>Onboard Temperature</t>
+  </si>
+  <si>
+    <t>BDPS MOSFET Temperature</t>
+  </si>
+  <si>
+    <t>Pre-Charge Resistors Temperature</t>
+  </si>
+  <si>
+    <t>Ambient Temperature</t>
+  </si>
+  <si>
+    <t>BCC IC Temperature</t>
+  </si>
+  <si>
+    <t>CELL_OV_FLT (CT overvoltage fault)</t>
+  </si>
+  <si>
+    <t>E-Num</t>
+  </si>
+  <si>
+    <t>CELL_UV_FLT (CT undervoltage fault)</t>
+  </si>
+  <si>
+    <t>CB_OPEN_FLT (Open CB fault)</t>
+  </si>
+  <si>
+    <t>CB_SHORT_FLT (Short CB fault)</t>
+  </si>
+  <si>
+    <t>GPIO_STS (GPIO status)</t>
+  </si>
+  <si>
+    <t>AN_OT_UT_FLT (AN over and undertemperature)</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>GPIO_SHORT_ANx_OPEN_STS (Short GPIO/open AN diagnostic)</t>
+  </si>
+  <si>
+    <t>COM_STATUS (Number of communication errors detected)</t>
+  </si>
+  <si>
+    <t>FAULT1_STATUS (Fault status)</t>
+  </si>
+  <si>
+    <t>FAULT2_STATUS (Fault status)</t>
+  </si>
+  <si>
+    <t>FAULT3_STATUS (Fault status)</t>
+  </si>
+  <si>
+    <t>Voltage</t>
+  </si>
+  <si>
+    <t>Bit-Fields</t>
+  </si>
+  <si>
+    <t>Algorithum Fault Status</t>
+  </si>
+  <si>
+    <t>uint8</t>
+  </si>
+  <si>
+    <t>BMS and FET Status</t>
+  </si>
+  <si>
+    <t>BMS Status</t>
+  </si>
+  <si>
+    <t>Cumulative Capacity</t>
+  </si>
+  <si>
+    <t>uint32</t>
+  </si>
+  <si>
+    <t>Ah</t>
+  </si>
+  <si>
+    <t>Algorithum</t>
+  </si>
+  <si>
+    <t>Cycle Count</t>
+  </si>
+  <si>
+    <t>SOC (OCV)</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>SOC (CC)</t>
+  </si>
+  <si>
+    <t>SOH</t>
   </si>
   <si>
     <t>bit_index</t>
@@ -222,9 +400,126 @@
     <t>inactive_text</t>
   </si>
   <si>
+    <t>Cell 1</t>
+  </si>
+  <si>
+    <t>ON</t>
+  </si>
+  <si>
+    <t>OFF</t>
+  </si>
+  <si>
+    <t>Cell 2</t>
+  </si>
+  <si>
+    <t>Cell 3</t>
+  </si>
+  <si>
+    <t>Cell 4</t>
+  </si>
+  <si>
+    <t>Cell 5</t>
+  </si>
+  <si>
+    <t>Cell 6</t>
+  </si>
+  <si>
+    <t>Cell 7</t>
+  </si>
+  <si>
+    <t>Cell 8</t>
+  </si>
+  <si>
+    <t>Cell 9</t>
+  </si>
+  <si>
+    <t>Cell 10</t>
+  </si>
+  <si>
+    <t>Cell 11</t>
+  </si>
+  <si>
+    <t>Cell 12</t>
+  </si>
+  <si>
+    <t>Cell 13</t>
+  </si>
+  <si>
+    <t>Cell 14</t>
+  </si>
+  <si>
+    <t>Cell Over Voltage (COV)</t>
+  </si>
+  <si>
+    <t>FAULT</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Cell Under Voltage (CUV)</t>
+  </si>
+  <si>
+    <t>Pack Over Voltage (POV)</t>
+  </si>
+  <si>
+    <t>Pack Under Voltage (PUV)</t>
+  </si>
+  <si>
+    <t>Voltage Sensing Mismatch</t>
+  </si>
+  <si>
+    <t>Over Current (OC)</t>
+  </si>
+  <si>
+    <t>Over Temperature (OT)</t>
+  </si>
+  <si>
+    <t>Under Temperature (UT)</t>
+  </si>
+  <si>
+    <t>Over-Discharge Protection (ODP)</t>
+  </si>
+  <si>
+    <t>Over Charge Protection (OCP)</t>
+  </si>
+  <si>
+    <t>Cell Voltage Imbalance</t>
+  </si>
+  <si>
+    <t>Thermal Imbalance</t>
+  </si>
+  <si>
+    <t>Main FET</t>
+  </si>
+  <si>
+    <t>Pre-Charge FET</t>
+  </si>
+  <si>
     <t>value</t>
   </si>
   <si>
+    <t>Rest</t>
+  </si>
+  <si>
+    <t>Discharge</t>
+  </si>
+  <si>
+    <t>Charge</t>
+  </si>
+  <si>
+    <t>group_name</t>
+  </si>
+  <si>
+    <t>operations</t>
+  </si>
+  <si>
+    <t>min|max|diff|avg</t>
+  </si>
+  <si>
+    <t>min|max|avg</t>
+  </si>
+  <si>
     <t>command_name</t>
   </si>
   <si>
@@ -240,274 +535,25 @@
     <t>timeout_ms</t>
   </si>
   <si>
-    <t>14 individual cell voltages expanded automatically</t>
-  </si>
-  <si>
-    <t>0x5000</t>
-  </si>
-  <si>
-    <t>Onboard Temperature Sensors</t>
-  </si>
-  <si>
-    <t>Pack Temperature Sensors</t>
-  </si>
-  <si>
-    <t>0x4000</t>
-  </si>
-  <si>
-    <t>Onboard Temperature</t>
-  </si>
-  <si>
-    <t>Pack Voltage &amp; Current</t>
-  </si>
-  <si>
-    <t>Balancing Resistor Temperature</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>BCC Fault Status</t>
-  </si>
-  <si>
-    <t>Array containing all fault status information provided by BCC</t>
-  </si>
-  <si>
-    <t>CELL_OV_FLT (CT overvoltage fault)</t>
-  </si>
-  <si>
-    <t>CELL_UV_FLT (CT undervoltage fault)</t>
-  </si>
-  <si>
-    <t>CB_OPEN_FLT (Open CB fault)</t>
-  </si>
-  <si>
-    <t>CB_SHORT_FLT (Short CB fault)</t>
-  </si>
-  <si>
-    <t>GPIO_STS (GPIO status)</t>
-  </si>
-  <si>
-    <t>AN_OT_UT_FLT (AN over and undertemperature)</t>
-  </si>
-  <si>
-    <t>GPIO_SHORT_ANx_OPEN_STS (Short GPIO/open AN diagnostic)</t>
-  </si>
-  <si>
-    <t>COM_STATUS (Number of communication errors detected)</t>
-  </si>
-  <si>
-    <t>FAULT1_STATUS (Fault status)</t>
-  </si>
-  <si>
-    <t>FAULT2_STATUS (Fault status)</t>
-  </si>
-  <si>
-    <t>FAULT3_STATUS (Fault status)</t>
-  </si>
-  <si>
-    <t>E-Num</t>
-  </si>
-  <si>
-    <t>big</t>
-  </si>
-  <si>
-    <t>uint32</t>
-  </si>
-  <si>
-    <t>int32</t>
-  </si>
-  <si>
-    <t>Series Cell Voltage</t>
-  </si>
-  <si>
-    <t>BCC IC Temperature</t>
-  </si>
-  <si>
-    <t>BDPS MOSFET Temperature</t>
-  </si>
-  <si>
-    <t>Pre-Charge Resistors Temperature</t>
-  </si>
-  <si>
-    <t>Ambient Temperature</t>
-  </si>
-  <si>
-    <t>0x6000</t>
-  </si>
-  <si>
-    <t>Load Voltage</t>
-  </si>
-  <si>
-    <t>Voltage</t>
-  </si>
-  <si>
-    <t>0x7000</t>
-  </si>
-  <si>
-    <t>0x8000</t>
-  </si>
-  <si>
-    <t>Fault Status</t>
-  </si>
-  <si>
-    <t>0x9000</t>
-  </si>
-  <si>
-    <t>Algorithum</t>
-  </si>
-  <si>
-    <t>Cell Balancing Status</t>
-  </si>
-  <si>
-    <t>Bit-Fields</t>
-  </si>
-  <si>
-    <t>BMS Status</t>
-  </si>
-  <si>
-    <t>uint8</t>
-  </si>
-  <si>
-    <t>FET Status</t>
-  </si>
-  <si>
-    <t>0x9001</t>
-  </si>
-  <si>
-    <t>Algorithm</t>
-  </si>
-  <si>
-    <t>Cumulative Capacity</t>
-  </si>
-  <si>
-    <t>Ah</t>
-  </si>
-  <si>
-    <t>Algorithum Fault Status</t>
-  </si>
-  <si>
-    <t>Cycle Count</t>
-  </si>
-  <si>
-    <t>SOC (OCV)</t>
-  </si>
-  <si>
-    <t>SOC (CC)</t>
-  </si>
-  <si>
-    <t>SOH</t>
-  </si>
-  <si>
-    <t>%</t>
-  </si>
-  <si>
-    <t>Cell 1</t>
-  </si>
-  <si>
-    <t>Cell 2</t>
-  </si>
-  <si>
-    <t>Cell 3</t>
-  </si>
-  <si>
-    <t>Cell 4</t>
-  </si>
-  <si>
-    <t>Cell 5</t>
-  </si>
-  <si>
-    <t>Cell 6</t>
-  </si>
-  <si>
-    <t>Cell 7</t>
-  </si>
-  <si>
-    <t>Cell 8</t>
-  </si>
-  <si>
-    <t>Cell 9</t>
-  </si>
-  <si>
-    <t>Cell 10</t>
-  </si>
-  <si>
-    <t>Cell 11</t>
-  </si>
-  <si>
-    <t>Cell 12</t>
-  </si>
-  <si>
-    <t>Cell 13</t>
-  </si>
-  <si>
-    <t>Cell 14</t>
-  </si>
-  <si>
-    <t>ON</t>
-  </si>
-  <si>
-    <t>OFF</t>
-  </si>
-  <si>
-    <t>Over Current (OC)</t>
-  </si>
-  <si>
-    <t>Pack Over Voltage (POV)</t>
-  </si>
-  <si>
-    <t>Cell Under Voltage (CUV)</t>
-  </si>
-  <si>
-    <t>Cell Over Voltage (COV)</t>
-  </si>
-  <si>
-    <t>Pack Under Voltage (PUV)</t>
-  </si>
-  <si>
-    <t>Over Charge Protection (OCP)</t>
-  </si>
-  <si>
-    <t>Over-Discharge Protection (ODP)</t>
-  </si>
-  <si>
-    <t>Cell Voltage Imbalance</t>
-  </si>
-  <si>
-    <t>Thermal Imbalance</t>
-  </si>
-  <si>
-    <t>Voltage Sensing Mismatch</t>
-  </si>
-  <si>
-    <t>Over Temperature (OT)</t>
-  </si>
-  <si>
-    <t>Under Temperature (UT)</t>
-  </si>
-  <si>
-    <t>FAULT</t>
-  </si>
-  <si>
-    <t>OK</t>
-  </si>
-  <si>
-    <t>Main FET</t>
-  </si>
-  <si>
-    <t>Pre-Charge FET</t>
-  </si>
-  <si>
-    <t>Discharge</t>
-  </si>
-  <si>
-    <t>Charge</t>
-  </si>
-  <si>
-    <t>Rest</t>
-  </si>
-  <si>
-    <t>BMS and FET Status</t>
+    <t>baud_rate</t>
+  </si>
+  <si>
+    <t>data_bits</t>
+  </si>
+  <si>
+    <t>stop_bits</t>
+  </si>
+  <si>
+    <t>parity</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>0x9002</t>
+  </si>
+  <si>
+    <t>BCC Status</t>
   </si>
 </sst>
 </file>
@@ -528,10 +574,9 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="8"/>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -569,11 +614,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -876,107 +922,188 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="11" customWidth="1"/>
-    <col min="4" max="4" width="12.90625" customWidth="1"/>
-    <col min="5" max="5" width="19.1796875" customWidth="1"/>
-    <col min="6" max="6" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.08984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.7265625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="20.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.36328125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.453125" customWidth="1"/>
+    <col min="17" max="17" width="13.1796875" customWidth="1"/>
+    <col min="19" max="19" width="7.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D2">
         <v>2</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2">
+        <v>23</v>
+      </c>
+      <c r="I2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2">
         <v>2</v>
       </c>
-      <c r="J2" t="s">
-        <v>89</v>
-      </c>
-      <c r="L2">
+      <c r="K2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P2">
         <v>10</v>
       </c>
-      <c r="M2">
+      <c r="Q2">
         <v>12</v>
       </c>
-      <c r="N2" t="s">
-        <v>20</v>
+      <c r="R2">
+        <v>1</v>
+      </c>
+      <c r="S2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>115200</v>
+      </c>
+      <c r="B2">
+        <v>8</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>172</v>
+      </c>
+      <c r="E2">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -986,7 +1113,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.54296875" bestFit="1" customWidth="1"/>
@@ -999,36 +1126,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="C2">
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -1036,16 +1163,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B3" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="C3">
         <v>28</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
@@ -1053,16 +1180,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="C4">
         <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -1070,16 +1197,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="C5">
         <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
@@ -1087,36 +1214,36 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="C6">
         <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>76</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>97</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="C7">
         <v>4</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
@@ -1124,16 +1251,16 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C8">
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
@@ -1141,16 +1268,16 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="C9">
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
@@ -1158,16 +1285,16 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>109</v>
+        <v>54</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -1175,18 +1302,35 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="B11" t="s">
-        <v>111</v>
+        <v>56</v>
       </c>
       <c r="C11">
         <v>13</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B12" t="s">
+        <v>174</v>
+      </c>
+      <c r="C12">
+        <v>25</v>
+      </c>
+      <c r="D12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1197,7 +1341,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
@@ -1214,63 +1358,63 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>31</v>
+        <v>58</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="N1" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F2">
         <v>1E-3</v>
@@ -1279,16 +1423,16 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="I2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J2" t="s">
         <v>72</v>
       </c>
-      <c r="J2" t="s">
-        <v>45</v>
-      </c>
       <c r="M2" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="N2" t="b">
         <v>1</v>
@@ -1296,19 +1440,19 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="C3" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F3">
         <v>1E-3</v>
@@ -1317,16 +1461,16 @@
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="I3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" t="s">
         <v>72</v>
       </c>
-      <c r="J3" t="s">
-        <v>45</v>
-      </c>
       <c r="M3" t="s">
-        <v>50</v>
+        <v>77</v>
       </c>
       <c r="N3" t="b">
         <v>1</v>
@@ -1334,19 +1478,19 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D4">
         <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F4">
         <v>1E-3</v>
@@ -1355,16 +1499,16 @@
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="I4" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="J4" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="M4" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
@@ -1372,19 +1516,19 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>81</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>82</v>
       </c>
       <c r="D5">
         <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F5">
         <v>0.1</v>
@@ -1393,16 +1537,16 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="I5" t="s">
-        <v>51</v>
+        <v>81</v>
       </c>
       <c r="J5" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="M5" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
@@ -1410,19 +1554,19 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="C6" t="s">
-        <v>48</v>
+        <v>82</v>
       </c>
       <c r="D6">
         <v>3</v>
       </c>
       <c r="E6" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F6">
         <v>0.1</v>
@@ -1431,16 +1575,16 @@
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="I6" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="J6" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="M6" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
@@ -1448,19 +1592,19 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="B7" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="C7" t="s">
-        <v>48</v>
+        <v>82</v>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F7">
         <v>0.1</v>
@@ -1469,16 +1613,16 @@
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="I7" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="J7" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="M7" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="N7" t="b">
         <v>1</v>
@@ -1486,19 +1630,19 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="C8" t="s">
-        <v>48</v>
+        <v>82</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F8">
         <v>0.1</v>
@@ -1507,16 +1651,16 @@
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="I8" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="J8" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="M8" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="N8" t="b">
         <v>1</v>
@@ -1524,19 +1668,19 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="B9" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>82</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F9">
         <v>0.1</v>
@@ -1545,16 +1689,16 @@
         <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="I9" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="J9" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="M9" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="N9" t="b">
         <v>1</v>
@@ -1562,19 +1706,19 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C10" t="s">
-        <v>48</v>
+        <v>82</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F10">
         <v>0.1</v>
@@ -1583,16 +1727,16 @@
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="I10" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="J10" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="M10" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="N10" t="b">
         <v>1</v>
@@ -1600,19 +1744,19 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D11">
         <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -1621,13 +1765,13 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I11" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="J11" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N11" t="b">
         <v>1</v>
@@ -1635,19 +1779,19 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B12" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D12">
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F12">
         <v>1</v>
@@ -1656,13 +1800,13 @@
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I12" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="J12" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N12" t="b">
         <v>1</v>
@@ -1670,19 +1814,19 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
       <c r="E13" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F13">
         <v>1</v>
@@ -1691,13 +1835,13 @@
         <v>0</v>
       </c>
       <c r="H13" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I13" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="J13" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N13" t="b">
         <v>1</v>
@@ -1705,19 +1849,19 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D14">
         <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F14">
         <v>1</v>
@@ -1726,13 +1870,13 @@
         <v>0</v>
       </c>
       <c r="H14" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I14" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="J14" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N14" t="b">
         <v>1</v>
@@ -1740,19 +1884,19 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B15" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="C15" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -1761,13 +1905,13 @@
         <v>0</v>
       </c>
       <c r="H15" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I15" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="J15" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N15" t="b">
         <v>1</v>
@@ -1775,19 +1919,19 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B16" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="C16" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F16">
         <v>1</v>
@@ -1796,16 +1940,16 @@
         <v>0</v>
       </c>
       <c r="H16" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I16" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="J16" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="M16" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="N16" t="b">
         <v>1</v>
@@ -1813,19 +1957,19 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B17" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="C17" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D17">
         <v>1</v>
       </c>
       <c r="E17" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F17">
         <v>1</v>
@@ -1834,13 +1978,13 @@
         <v>0</v>
       </c>
       <c r="H17" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I17" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="J17" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N17" t="b">
         <v>1</v>
@@ -1848,19 +1992,19 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B18" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="C18" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
       <c r="E18" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F18">
         <v>1</v>
@@ -1869,13 +2013,13 @@
         <v>0</v>
       </c>
       <c r="H18" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I18" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="J18" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N18" t="b">
         <v>1</v>
@@ -1883,19 +2027,19 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B19" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="C19" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D19">
         <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F19">
         <v>1</v>
@@ -1904,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="H19" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I19" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="J19" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N19" t="b">
         <v>1</v>
@@ -1918,19 +2062,19 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B20" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="C20" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D20">
         <v>1</v>
       </c>
       <c r="E20" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -1939,13 +2083,13 @@
         <v>0</v>
       </c>
       <c r="H20" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I20" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="J20" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N20" t="b">
         <v>1</v>
@@ -1953,19 +2097,19 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B21" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="C21" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D21">
         <v>1</v>
       </c>
       <c r="E21" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F21">
         <v>1</v>
@@ -1974,13 +2118,13 @@
         <v>0</v>
       </c>
       <c r="H21" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I21" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="J21" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N21" t="b">
         <v>1</v>
@@ -1988,19 +2132,19 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>97</v>
+        <v>47</v>
       </c>
       <c r="B22" t="s">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="C22" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="D22">
         <v>1</v>
       </c>
       <c r="E22" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F22">
         <v>9.9999999999999995E-7</v>
@@ -2009,13 +2153,13 @@
         <v>0</v>
       </c>
       <c r="H22" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="I22" t="s">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="J22" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N22" t="b">
         <v>1</v>
@@ -2023,19 +2167,19 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B23" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C23" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D23">
         <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F23">
         <v>1</v>
@@ -2044,13 +2188,13 @@
         <v>0</v>
       </c>
       <c r="H23" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I23" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="J23" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N23" t="b">
         <v>1</v>
@@ -2058,19 +2202,19 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B24" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="C24" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D24">
         <v>1</v>
       </c>
       <c r="E24" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F24">
         <v>1</v>
@@ -2079,13 +2223,13 @@
         <v>0</v>
       </c>
       <c r="H24" t="s">
+        <v>105</v>
+      </c>
+      <c r="I24" t="s">
         <v>106</v>
       </c>
-      <c r="I24" t="s">
-        <v>114</v>
-      </c>
       <c r="J24" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N24" t="b">
         <v>1</v>
@@ -2093,19 +2237,19 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="B25" t="s">
-        <v>109</v>
+        <v>54</v>
       </c>
       <c r="C25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D25">
         <v>1</v>
       </c>
       <c r="E25" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F25">
         <v>1</v>
@@ -2114,13 +2258,13 @@
         <v>0</v>
       </c>
       <c r="H25" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I25" t="s">
-        <v>155</v>
+        <v>108</v>
       </c>
       <c r="J25" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N25" t="b">
         <v>1</v>
@@ -2128,19 +2272,19 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="B26" t="s">
+        <v>109</v>
+      </c>
+      <c r="C26" t="s">
         <v>107</v>
       </c>
-      <c r="C26" t="s">
-        <v>108</v>
-      </c>
       <c r="D26">
         <v>1</v>
       </c>
       <c r="E26" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F26">
         <v>1</v>
@@ -2149,13 +2293,13 @@
         <v>0</v>
       </c>
       <c r="H26" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I26" t="s">
-        <v>155</v>
+        <v>108</v>
       </c>
       <c r="J26" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N26" t="b">
         <v>1</v>
@@ -2163,19 +2307,19 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" t="s">
         <v>110</v>
       </c>
-      <c r="B27" t="s">
-        <v>112</v>
-      </c>
       <c r="C27" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="D27">
         <v>1</v>
       </c>
       <c r="E27" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F27">
         <v>1</v>
@@ -2184,13 +2328,13 @@
         <v>0</v>
       </c>
       <c r="H27" t="s">
+        <v>112</v>
+      </c>
+      <c r="I27" t="s">
         <v>113</v>
       </c>
-      <c r="I27" t="s">
-        <v>104</v>
-      </c>
       <c r="J27" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N27" t="b">
         <v>1</v>
@@ -2198,19 +2342,19 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="B28" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C28" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D28">
         <v>1</v>
       </c>
       <c r="E28" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -2219,13 +2363,13 @@
         <v>0</v>
       </c>
       <c r="H28" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="I28" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="J28" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N28" t="b">
         <v>1</v>
@@ -2233,19 +2377,19 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="B29" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C29" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D29">
         <v>1</v>
       </c>
       <c r="E29" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F29">
         <v>0.01</v>
@@ -2254,13 +2398,13 @@
         <v>0</v>
       </c>
       <c r="H29" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I29" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="J29" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N29" t="b">
         <v>1</v>
@@ -2268,19 +2412,19 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="B30" t="s">
         <v>117</v>
       </c>
       <c r="C30" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D30">
         <v>1</v>
       </c>
       <c r="E30" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F30">
         <v>1</v>
@@ -2289,13 +2433,13 @@
         <v>0</v>
       </c>
       <c r="H30" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I30" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="J30" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N30" t="b">
         <v>1</v>
@@ -2303,19 +2447,19 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="B31" t="s">
         <v>118</v>
       </c>
       <c r="C31" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="D31">
         <v>1</v>
       </c>
       <c r="E31" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F31">
         <v>0.01</v>
@@ -2324,22 +2468,56 @@
         <v>0</v>
       </c>
       <c r="H31" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I31" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="J31" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="N31" t="b">
         <v>1</v>
       </c>
     </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>173</v>
+      </c>
+      <c r="B32" t="s">
+        <v>174</v>
+      </c>
+      <c r="C32" t="s">
+        <v>107</v>
+      </c>
+      <c r="D32">
+        <v>25</v>
+      </c>
+      <c r="E32" t="s">
+        <v>22</v>
+      </c>
+      <c r="F32">
+        <v>1</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
+      <c r="H32" t="s">
+        <v>92</v>
+      </c>
+      <c r="I32" t="s">
+        <v>174</v>
+      </c>
+      <c r="J32" t="s">
+        <v>72</v>
+      </c>
+      <c r="N32" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
@@ -2358,310 +2536,310 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>31</v>
+        <v>58</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>119</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>57</v>
+        <v>120</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>58</v>
+        <v>121</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>59</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E2" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F2" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="E3" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F3" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="E4" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F4" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C5">
         <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E5" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F5" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C6">
         <v>4</v>
       </c>
       <c r="D6" t="s">
+        <v>129</v>
+      </c>
+      <c r="E6" t="s">
         <v>124</v>
       </c>
-      <c r="E6" t="s">
-        <v>134</v>
-      </c>
       <c r="F6" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C7">
         <v>5</v>
       </c>
       <c r="D7" t="s">
+        <v>130</v>
+      </c>
+      <c r="E7" t="s">
+        <v>124</v>
+      </c>
+      <c r="F7" t="s">
         <v>125</v>
-      </c>
-      <c r="E7" t="s">
-        <v>134</v>
-      </c>
-      <c r="F7" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C8">
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="E8" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F8" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C9">
         <v>7</v>
       </c>
       <c r="D9" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="E9" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F9" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B10" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C10">
         <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="E10" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F10" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C11">
         <v>9</v>
       </c>
       <c r="D11" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="E11" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F11" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B12" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C12">
         <v>10</v>
       </c>
       <c r="D12" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="E12" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F12" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B13" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C13">
         <v>11</v>
       </c>
       <c r="D13" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="E13" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F13" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B14" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C14">
         <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="E14" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F14" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B15" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="C15">
         <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="E15" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F15" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B16" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -2670,78 +2848,78 @@
         <v>139</v>
       </c>
       <c r="E16" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F16" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B17" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="E17" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F17" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B18" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="E18" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F18" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B19" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19" t="s">
+        <v>144</v>
+      </c>
+      <c r="E19" t="s">
         <v>140</v>
       </c>
-      <c r="E19" t="s">
-        <v>148</v>
-      </c>
       <c r="F19" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B20" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="C20">
         <v>4</v>
@@ -2750,194 +2928,193 @@
         <v>145</v>
       </c>
       <c r="E20" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F20" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B21" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="C21">
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="E21" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F21" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B22" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="C22">
         <v>6</v>
       </c>
       <c r="D22" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E22" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F22" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B23" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="C23">
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E23" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F23" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B24" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="C24">
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="E24" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F24" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B25" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="C25">
         <v>9</v>
       </c>
       <c r="D25" t="s">
+        <v>150</v>
+      </c>
+      <c r="E25" t="s">
+        <v>140</v>
+      </c>
+      <c r="F25" t="s">
         <v>141</v>
-      </c>
-      <c r="E25" t="s">
-        <v>148</v>
-      </c>
-      <c r="F25" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B26" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="C26">
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="E26" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F26" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B27" t="s">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="C27">
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="E27" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F27" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="B28" t="s">
-        <v>109</v>
+        <v>54</v>
       </c>
       <c r="C28">
         <v>0</v>
       </c>
       <c r="D28" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E28" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F28" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="B29" t="s">
-        <v>109</v>
+        <v>54</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="E29" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F29" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2955,68 +3132,149 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>31</v>
+        <v>58</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>60</v>
+        <v>155</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>57</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" t="s">
+        <v>162</v>
+      </c>
+      <c r="C4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -3029,19 +3287,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>163</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>62</v>
+        <v>164</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -3049,8 +3307,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -3068,34 +3326,34 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="E1" s="1" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>37</v>
+        <v>64</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>40</v>
+        <v>67</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>63</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -3103,9 +3361,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:D11"/>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
@@ -3116,21 +3374,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>64</v>
+        <v>166</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>167</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B2">
         <v>500</v>
@@ -3144,7 +3402,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B3">
         <v>500</v>
@@ -3158,7 +3416,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="B4">
         <v>500</v>
@@ -3172,7 +3430,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="B5">
         <v>500</v>
@@ -3186,7 +3444,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B6">
         <v>500</v>
@@ -3200,7 +3458,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>97</v>
+        <v>47</v>
       </c>
       <c r="B7">
         <v>500</v>
@@ -3214,7 +3472,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="B8">
         <v>500</v>
@@ -3228,7 +3486,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="B9">
         <v>500</v>
@@ -3242,7 +3500,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="B10">
         <v>500</v>
@@ -3256,7 +3514,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="B11">
         <v>500</v>
@@ -3268,8 +3526,21 @@
         <v>1</v>
       </c>
     </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B12">
+        <v>500</v>
+      </c>
+      <c r="C12">
+        <v>500</v>
+      </c>
+      <c r="D12" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>